<commit_message>
Update for Final claimant level Summary
</commit_message>
<xml_diff>
--- a/data/05_claimant_multi.xlsx
+++ b/data/05_claimant_multi.xlsx
@@ -501,7 +501,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>94.70775168837672</v>
+        <v>94.7077516883767</v>
       </c>
       <c r="J2" t="n">
         <v>4</v>
@@ -649,7 +649,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>60.9797629494325</v>
+        <v>60.97976294943251</v>
       </c>
       <c r="J6" t="n">
         <v>4</v>
@@ -686,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>54.78528270852915</v>
+        <v>54.78528270852914</v>
       </c>
       <c r="J7" t="n">
         <v>4</v>
@@ -723,7 +723,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>45.08863202851241</v>
+        <v>45.08863202851243</v>
       </c>
       <c r="J8" t="n">
         <v>4</v>
@@ -797,7 +797,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>46.50357359488781</v>
+        <v>46.5035735948878</v>
       </c>
       <c r="J10" t="n">
         <v>4</v>
@@ -834,7 +834,7 @@
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>41.21814719090343</v>
+        <v>41.21814719090342</v>
       </c>
       <c r="J11" t="n">
         <v>4</v>
@@ -908,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>47.82037460761672</v>
+        <v>47.82037460761673</v>
       </c>
       <c r="J13" t="n">
         <v>4</v>
@@ -982,7 +982,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>58.29437574506219</v>
+        <v>58.2943757450622</v>
       </c>
       <c r="J15" t="n">
         <v>4</v>
@@ -1056,7 +1056,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>48.80990131814055</v>
+        <v>48.80990131814056</v>
       </c>
       <c r="J17" t="n">
         <v>4</v>
@@ -6421,7 +6421,7 @@
         <v>0</v>
       </c>
       <c r="I162" t="n">
-        <v>15.19855939370729</v>
+        <v>15.19855939370728</v>
       </c>
       <c r="J162" t="n">
         <v>0</v>
@@ -8715,7 +8715,7 @@
         <v>0</v>
       </c>
       <c r="I224" t="n">
-        <v>21.68485392803642</v>
+        <v>21.68485392803641</v>
       </c>
       <c r="J224" t="n">
         <v>0</v>
@@ -9566,7 +9566,7 @@
         <v>0</v>
       </c>
       <c r="I247" t="n">
-        <v>10.50323123245468</v>
+        <v>10.50323123245469</v>
       </c>
       <c r="J247" t="n">
         <v>0</v>
@@ -9788,7 +9788,7 @@
         <v>0</v>
       </c>
       <c r="I253" t="n">
-        <v>5.367032133328139</v>
+        <v>5.36703213332814</v>
       </c>
       <c r="J253" t="n">
         <v>1</v>
@@ -10232,7 +10232,7 @@
         <v>0</v>
       </c>
       <c r="I265" t="n">
-        <v>5.718760806012174</v>
+        <v>5.718760806012175</v>
       </c>
       <c r="J265" t="n">
         <v>0</v>
@@ -11416,7 +11416,7 @@
         <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>17.26530482728611</v>
+        <v>17.2653048272861</v>
       </c>
       <c r="J297" t="n">
         <v>0</v>
@@ -11490,7 +11490,7 @@
         <v>0</v>
       </c>
       <c r="I299" t="n">
-        <v>5.963783319973528</v>
+        <v>5.963783319973527</v>
       </c>
       <c r="J299" t="n">
         <v>0</v>
@@ -13155,7 +13155,7 @@
         <v>0</v>
       </c>
       <c r="I344" t="n">
-        <v>3.685890433178162</v>
+        <v>3.685890433178163</v>
       </c>
       <c r="J344" t="n">
         <v>0</v>
@@ -15745,7 +15745,7 @@
         <v>0</v>
       </c>
       <c r="I414" t="n">
-        <v>8.517749253008612</v>
+        <v>8.51774925300861</v>
       </c>
       <c r="J414" t="n">
         <v>0</v>
@@ -16744,7 +16744,7 @@
         <v>0</v>
       </c>
       <c r="I441" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J441" t="n">
         <v>0</v>
@@ -16781,7 +16781,7 @@
         <v>0</v>
       </c>
       <c r="I442" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J442" t="n">
         <v>0</v>
@@ -16818,7 +16818,7 @@
         <v>0</v>
       </c>
       <c r="I443" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J443" t="n">
         <v>0</v>
@@ -16855,7 +16855,7 @@
         <v>0</v>
       </c>
       <c r="I444" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J444" t="n">
         <v>0</v>
@@ -16892,7 +16892,7 @@
         <v>0</v>
       </c>
       <c r="I445" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J445" t="n">
         <v>0</v>
@@ -16929,7 +16929,7 @@
         <v>0</v>
       </c>
       <c r="I446" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J446" t="n">
         <v>0</v>
@@ -16966,7 +16966,7 @@
         <v>0</v>
       </c>
       <c r="I447" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J447" t="n">
         <v>0</v>
@@ -17003,7 +17003,7 @@
         <v>0</v>
       </c>
       <c r="I448" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J448" t="n">
         <v>0</v>
@@ -17040,7 +17040,7 @@
         <v>0</v>
       </c>
       <c r="I449" t="n">
-        <v>4.181903936763551</v>
+        <v>4.181903936763552</v>
       </c>
       <c r="J449" t="n">
         <v>0</v>
@@ -17077,7 +17077,7 @@
         <v>0</v>
       </c>
       <c r="I450" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J450" t="n">
         <v>0</v>
@@ -17114,7 +17114,7 @@
         <v>0</v>
       </c>
       <c r="I451" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J451" t="n">
         <v>0</v>
@@ -17151,7 +17151,7 @@
         <v>0</v>
       </c>
       <c r="I452" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J452" t="n">
         <v>0</v>
@@ -17188,7 +17188,7 @@
         <v>0</v>
       </c>
       <c r="I453" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J453" t="n">
         <v>0</v>
@@ -17225,7 +17225,7 @@
         <v>0</v>
       </c>
       <c r="I454" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J454" t="n">
         <v>0</v>
@@ -17262,7 +17262,7 @@
         <v>0</v>
       </c>
       <c r="I455" t="n">
-        <v>4.356331944470609</v>
+        <v>4.35633194447061</v>
       </c>
       <c r="J455" t="n">
         <v>0</v>
@@ -22886,7 +22886,7 @@
         <v>0</v>
       </c>
       <c r="I607" t="n">
-        <v>3.582200816652933</v>
+        <v>3.582200816652934</v>
       </c>
       <c r="J607" t="n">
         <v>0</v>
@@ -23663,7 +23663,7 @@
         <v>0</v>
       </c>
       <c r="I628" t="n">
-        <v>3.746605840067305</v>
+        <v>3.746605840067306</v>
       </c>
       <c r="J628" t="n">
         <v>0</v>
@@ -24440,7 +24440,7 @@
         <v>0</v>
       </c>
       <c r="I649" t="n">
-        <v>3.084359591344127</v>
+        <v>3.084359591344128</v>
       </c>
       <c r="J649" t="n">
         <v>0</v>
@@ -24995,7 +24995,7 @@
         <v>0</v>
       </c>
       <c r="I664" t="n">
-        <v>3.547173846867319</v>
+        <v>3.54717384686732</v>
       </c>
       <c r="J664" t="n">
         <v>0</v>
@@ -25032,7 +25032,7 @@
         <v>0</v>
       </c>
       <c r="I665" t="n">
-        <v>3.547173846867319</v>
+        <v>3.54717384686732</v>
       </c>
       <c r="J665" t="n">
         <v>0</v>
@@ -25069,7 +25069,7 @@
         <v>0</v>
       </c>
       <c r="I666" t="n">
-        <v>3.547173846867319</v>
+        <v>3.54717384686732</v>
       </c>
       <c r="J666" t="n">
         <v>0</v>
@@ -25106,7 +25106,7 @@
         <v>0</v>
       </c>
       <c r="I667" t="n">
-        <v>3.547173846867319</v>
+        <v>3.54717384686732</v>
       </c>
       <c r="J667" t="n">
         <v>0</v>
@@ -25143,7 +25143,7 @@
         <v>0</v>
       </c>
       <c r="I668" t="n">
-        <v>3.547173846867319</v>
+        <v>3.54717384686732</v>
       </c>
       <c r="J668" t="n">
         <v>0</v>
@@ -27622,7 +27622,7 @@
         <v>0</v>
       </c>
       <c r="I735" t="n">
-        <v>4.561302586247236</v>
+        <v>4.561302586247237</v>
       </c>
       <c r="J735" t="n">
         <v>0</v>
@@ -27696,7 +27696,7 @@
         <v>0</v>
       </c>
       <c r="I737" t="n">
-        <v>4.232281202690739</v>
+        <v>4.23228120269074</v>
       </c>
       <c r="J737" t="n">
         <v>0</v>
@@ -30138,7 +30138,7 @@
         <v>0</v>
       </c>
       <c r="I803" t="n">
-        <v>3.579088029987331</v>
+        <v>3.57908802998733</v>
       </c>
       <c r="J803" t="n">
         <v>0</v>
@@ -31063,7 +31063,7 @@
         <v>0</v>
       </c>
       <c r="I828" t="n">
-        <v>2.922796490713548</v>
+        <v>2.922796490713549</v>
       </c>
       <c r="J828" t="n">
         <v>0</v>
@@ -31433,7 +31433,7 @@
         <v>0</v>
       </c>
       <c r="I838" t="n">
-        <v>2.967757702304283</v>
+        <v>2.967757702304284</v>
       </c>
       <c r="J838" t="n">
         <v>0</v>
@@ -31803,7 +31803,7 @@
         <v>0</v>
       </c>
       <c r="I848" t="n">
-        <v>2.588617298338555</v>
+        <v>2.588617298338556</v>
       </c>
       <c r="J848" t="n">
         <v>0</v>
@@ -31914,7 +31914,7 @@
         <v>0</v>
       </c>
       <c r="I851" t="n">
-        <v>3.061794556124312</v>
+        <v>3.061794556124313</v>
       </c>
       <c r="J851" t="n">
         <v>0</v>
@@ -32247,7 +32247,7 @@
         <v>0</v>
       </c>
       <c r="I860" t="n">
-        <v>3.49113846783982</v>
+        <v>3.491138467839821</v>
       </c>
       <c r="J860" t="n">
         <v>0</v>
@@ -33986,7 +33986,7 @@
         <v>0</v>
       </c>
       <c r="I907" t="n">
-        <v>4.106042677208306</v>
+        <v>4.106042677208307</v>
       </c>
       <c r="J907" t="n">
         <v>0</v>
@@ -34245,7 +34245,7 @@
         <v>0</v>
       </c>
       <c r="I914" t="n">
-        <v>3.701074627783834</v>
+        <v>3.701074627783833</v>
       </c>
       <c r="J914" t="n">
         <v>0</v>
@@ -34504,7 +34504,7 @@
         <v>0</v>
       </c>
       <c r="I921" t="n">
-        <v>4.113657565336344</v>
+        <v>4.113657565336345</v>
       </c>
       <c r="J921" t="n">
         <v>0</v>
@@ -35392,7 +35392,7 @@
         <v>0</v>
       </c>
       <c r="I945" t="n">
-        <v>4.208315352651369</v>
+        <v>4.20831535265137</v>
       </c>
       <c r="J945" t="n">
         <v>0</v>
@@ -37131,7 +37131,7 @@
         <v>0</v>
       </c>
       <c r="I992" t="n">
-        <v>4.190014814242932</v>
+        <v>4.190014814242933</v>
       </c>
       <c r="J992" t="n">
         <v>0</v>
@@ -37205,7 +37205,7 @@
         <v>0</v>
       </c>
       <c r="I994" t="n">
-        <v>4.769300912985992</v>
+        <v>4.769300912985993</v>
       </c>
       <c r="J994" t="n">
         <v>0</v>
@@ -38352,7 +38352,7 @@
         <v>0</v>
       </c>
       <c r="I1025" t="n">
-        <v>4.121256462165123</v>
+        <v>4.121256462165124</v>
       </c>
       <c r="J1025" t="n">
         <v>0</v>
@@ -39499,7 +39499,7 @@
         <v>0</v>
       </c>
       <c r="I1056" t="n">
-        <v>4.387651886525599</v>
+        <v>4.387651886525598</v>
       </c>
       <c r="J1056" t="n">
         <v>0</v>
@@ -40683,7 +40683,7 @@
         <v>0</v>
       </c>
       <c r="I1088" t="n">
-        <v>4.170431333572302</v>
+        <v>4.170431333572303</v>
       </c>
       <c r="J1088" t="n">
         <v>0</v>
@@ -40831,7 +40831,7 @@
         <v>0</v>
       </c>
       <c r="I1092" t="n">
-        <v>4.14917835988296</v>
+        <v>4.149178359882961</v>
       </c>
       <c r="J1092" t="n">
         <v>0</v>
@@ -40905,7 +40905,7 @@
         <v>0</v>
       </c>
       <c r="I1094" t="n">
-        <v>4.165074598860803</v>
+        <v>4.165074598860804</v>
       </c>
       <c r="J1094" t="n">
         <v>0</v>
@@ -41127,7 +41127,7 @@
         <v>0</v>
       </c>
       <c r="I1100" t="n">
-        <v>4.151425366146588</v>
+        <v>4.151425366146589</v>
       </c>
       <c r="J1100" t="n">
         <v>0</v>
@@ -41238,7 +41238,7 @@
         <v>0</v>
       </c>
       <c r="I1103" t="n">
-        <v>4.160549045041108</v>
+        <v>4.160549045041109</v>
       </c>
       <c r="J1103" t="n">
         <v>0</v>
@@ -42755,7 +42755,7 @@
         <v>0</v>
       </c>
       <c r="I1144" t="n">
-        <v>4.141098323576253</v>
+        <v>4.141098323576254</v>
       </c>
       <c r="J1144" t="n">
         <v>0</v>
@@ -43495,7 +43495,7 @@
         <v>0</v>
       </c>
       <c r="I1164" t="n">
-        <v>3.145740248392617</v>
+        <v>3.145740248392618</v>
       </c>
       <c r="J1164" t="n">
         <v>0</v>
@@ -43569,7 +43569,7 @@
         <v>0</v>
       </c>
       <c r="I1166" t="n">
-        <v>3.250834996693371</v>
+        <v>3.250834996693372</v>
       </c>
       <c r="J1166" t="n">
         <v>0</v>
@@ -44272,7 +44272,7 @@
         <v>0</v>
       </c>
       <c r="I1185" t="n">
-        <v>2.452524709325937</v>
+        <v>2.452524709325938</v>
       </c>
       <c r="J1185" t="n">
         <v>0</v>
@@ -44790,7 +44790,7 @@
         <v>0</v>
       </c>
       <c r="I1199" t="n">
-        <v>2.761598869876469</v>
+        <v>2.76159886987647</v>
       </c>
       <c r="J1199" t="n">
         <v>0</v>
@@ -44827,7 +44827,7 @@
         <v>0</v>
       </c>
       <c r="I1200" t="n">
-        <v>3.014687475234173</v>
+        <v>3.014687475234174</v>
       </c>
       <c r="J1200" t="n">
         <v>0</v>
@@ -47121,7 +47121,7 @@
         <v>0</v>
       </c>
       <c r="I1262" t="n">
-        <v>2.998488147058784</v>
+        <v>2.998488147058785</v>
       </c>
       <c r="J1262" t="n">
         <v>0</v>
@@ -47454,7 +47454,7 @@
         <v>0</v>
       </c>
       <c r="I1271" t="n">
-        <v>3.355918490649331</v>
+        <v>3.355918490649332</v>
       </c>
       <c r="J1271" t="n">
         <v>0</v>
@@ -47935,7 +47935,7 @@
         <v>0</v>
       </c>
       <c r="I1284" t="n">
-        <v>2.992047409941502</v>
+        <v>2.992047409941503</v>
       </c>
       <c r="J1284" t="n">
         <v>0</v>
@@ -48157,7 +48157,7 @@
         <v>0</v>
       </c>
       <c r="I1290" t="n">
-        <v>3.082862913468468</v>
+        <v>3.082862913468469</v>
       </c>
       <c r="J1290" t="n">
         <v>0</v>
@@ -49156,7 +49156,7 @@
         <v>0</v>
       </c>
       <c r="I1317" t="n">
-        <v>3.037007107876362</v>
+        <v>3.037007107876363</v>
       </c>
       <c r="J1317" t="n">
         <v>0</v>
@@ -50192,7 +50192,7 @@
         <v>0</v>
       </c>
       <c r="I1345" t="n">
-        <v>3.044039009134857</v>
+        <v>3.044039009134858</v>
       </c>
       <c r="J1345" t="n">
         <v>0</v>
@@ -50673,7 +50673,7 @@
         <v>0</v>
       </c>
       <c r="I1358" t="n">
-        <v>3.15814738946925</v>
+        <v>3.158147389469251</v>
       </c>
       <c r="J1358" t="n">
         <v>0</v>
@@ -50821,7 +50821,7 @@
         <v>0</v>
       </c>
       <c r="I1362" t="n">
-        <v>3.214655378858435</v>
+        <v>3.214655378858436</v>
       </c>
       <c r="J1362" t="n">
         <v>0</v>
@@ -51524,7 +51524,7 @@
         <v>0</v>
       </c>
       <c r="I1381" t="n">
-        <v>3.248705653166036</v>
+        <v>3.248705653166037</v>
       </c>
       <c r="J1381" t="n">
         <v>0</v>
@@ -51894,7 +51894,7 @@
         <v>0</v>
       </c>
       <c r="I1391" t="n">
-        <v>3.173236058942925</v>
+        <v>3.173236058942926</v>
       </c>
       <c r="J1391" t="n">
         <v>0</v>
@@ -52819,7 +52819,7 @@
         <v>0</v>
       </c>
       <c r="I1416" t="n">
-        <v>2.62414975751912</v>
+        <v>2.624149757519121</v>
       </c>
       <c r="J1416" t="n">
         <v>0</v>
@@ -53226,7 +53226,7 @@
         <v>0</v>
       </c>
       <c r="I1427" t="n">
-        <v>3.101012353081095</v>
+        <v>3.101012353081096</v>
       </c>
       <c r="J1427" t="n">
         <v>0</v>
@@ -53374,7 +53374,7 @@
         <v>0</v>
       </c>
       <c r="I1431" t="n">
-        <v>2.990702753686435</v>
+        <v>2.990702753686436</v>
       </c>
       <c r="J1431" t="n">
         <v>0</v>
@@ -54299,7 +54299,7 @@
         <v>0</v>
       </c>
       <c r="I1456" t="n">
-        <v>3.089480401964206</v>
+        <v>3.089480401964207</v>
       </c>
       <c r="J1456" t="n">
         <v>0</v>
@@ -57074,7 +57074,7 @@
         <v>0</v>
       </c>
       <c r="I1531" t="n">
-        <v>3.185554364047797</v>
+        <v>3.185554364047798</v>
       </c>
       <c r="J1531" t="n">
         <v>0</v>
@@ -58184,7 +58184,7 @@
         <v>0</v>
       </c>
       <c r="I1561" t="n">
-        <v>3.059607470800078</v>
+        <v>3.059607470800079</v>
       </c>
       <c r="J1561" t="n">
         <v>0</v>
@@ -59109,7 +59109,7 @@
         <v>0</v>
       </c>
       <c r="I1586" t="n">
-        <v>3.778922134967482</v>
+        <v>3.778922134967483</v>
       </c>
       <c r="J1586" t="n">
         <v>0</v>
@@ -61551,7 +61551,7 @@
         <v>0</v>
       </c>
       <c r="I1652" t="n">
-        <v>3.025846347313155</v>
+        <v>3.025846347313156</v>
       </c>
       <c r="J1652" t="n">
         <v>0</v>
@@ -61847,7 +61847,7 @@
         <v>0</v>
       </c>
       <c r="I1660" t="n">
-        <v>3.059577568281114</v>
+        <v>3.059577568281115</v>
       </c>
       <c r="J1660" t="n">
         <v>0</v>
@@ -62180,7 +62180,7 @@
         <v>0</v>
       </c>
       <c r="I1669" t="n">
-        <v>3.064381133041122</v>
+        <v>3.064381133041123</v>
       </c>
       <c r="J1669" t="n">
         <v>0</v>
@@ -62217,7 +62217,7 @@
         <v>0</v>
       </c>
       <c r="I1670" t="n">
-        <v>2.995013602268597</v>
+        <v>2.995013602268598</v>
       </c>
       <c r="J1670" t="n">
         <v>0</v>
@@ -63697,7 +63697,7 @@
         <v>0</v>
       </c>
       <c r="I1710" t="n">
-        <v>3.053903190131124</v>
+        <v>3.053903190131125</v>
       </c>
       <c r="J1710" t="n">
         <v>0</v>
@@ -65991,7 +65991,7 @@
         <v>0</v>
       </c>
       <c r="I1772" t="n">
-        <v>2.774704707782978</v>
+        <v>2.774704707782979</v>
       </c>
       <c r="J1772" t="n">
         <v>0</v>
@@ -66916,7 +66916,7 @@
         <v>0</v>
       </c>
       <c r="I1797" t="n">
-        <v>2.466522740639988</v>
+        <v>2.466522740639987</v>
       </c>
       <c r="J1797" t="n">
         <v>0</v>
@@ -67101,7 +67101,7 @@
         <v>0</v>
       </c>
       <c r="I1802" t="n">
-        <v>3.079958546686898</v>
+        <v>3.079958546686897</v>
       </c>
       <c r="J1802" t="n">
         <v>0</v>
@@ -68766,7 +68766,7 @@
         <v>0</v>
       </c>
       <c r="I1847" t="n">
-        <v>2.250342159302003</v>
+        <v>2.250342159302004</v>
       </c>
       <c r="J1847" t="n">
         <v>0</v>
@@ -69210,7 +69210,7 @@
         <v>0</v>
       </c>
       <c r="I1859" t="n">
-        <v>2.971567004180068</v>
+        <v>2.971567004180069</v>
       </c>
       <c r="J1859" t="n">
         <v>0</v>
@@ -69284,7 +69284,7 @@
         <v>0</v>
       </c>
       <c r="I1861" t="n">
-        <v>3.000365135167034</v>
+        <v>3.000365135167035</v>
       </c>
       <c r="J1861" t="n">
         <v>0</v>
@@ -69839,7 +69839,7 @@
         <v>0</v>
       </c>
       <c r="I1876" t="n">
-        <v>2.906838974461198</v>
+        <v>2.906838974461199</v>
       </c>
       <c r="J1876" t="n">
         <v>0</v>
@@ -70468,7 +70468,7 @@
         <v>0</v>
       </c>
       <c r="I1893" t="n">
-        <v>4.393097699449738</v>
+        <v>4.393097699449737</v>
       </c>
       <c r="J1893" t="n">
         <v>0</v>
@@ -70727,7 +70727,7 @@
         <v>0</v>
       </c>
       <c r="I1900" t="n">
-        <v>2.963449295919439</v>
+        <v>2.96344929591944</v>
       </c>
       <c r="J1900" t="n">
         <v>0</v>
@@ -71097,7 +71097,7 @@
         <v>0</v>
       </c>
       <c r="I1910" t="n">
-        <v>7.69817784444504</v>
+        <v>7.698177844445039</v>
       </c>
       <c r="J1910" t="n">
         <v>0</v>
@@ -71208,7 +71208,7 @@
         <v>0</v>
       </c>
       <c r="I1913" t="n">
-        <v>3.377997320867158</v>
+        <v>3.377997320867157</v>
       </c>
       <c r="J1913" t="n">
         <v>0</v>
@@ -71245,7 +71245,7 @@
         <v>0</v>
       </c>
       <c r="I1914" t="n">
-        <v>4.243292234653978</v>
+        <v>4.243292234653977</v>
       </c>
       <c r="J1914" t="n">
         <v>0</v>
@@ -71985,7 +71985,7 @@
         <v>0</v>
       </c>
       <c r="I1934" t="n">
-        <v>4.008230058747661</v>
+        <v>4.00823005874766</v>
       </c>
       <c r="J1934" t="n">
         <v>0</v>
@@ -72355,7 +72355,7 @@
         <v>0</v>
       </c>
       <c r="I1944" t="n">
-        <v>2.462219834808299</v>
+        <v>2.462219834808298</v>
       </c>
       <c r="J1944" t="n">
         <v>0</v>

</xml_diff>